<commit_message>
Add hero-article block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (9):
- blocks/hero-article/hero-article.css
- blocks/hero-article/hero-article.js
- drafts/us/en/news/featured-stories/2025/06/get-ahead-with-energy-storage-or-risk-getting-left-behind.plain.html
- tools/importer/import-featured-story.bundle.js
- tools/importer/import-featured-story.js
- tools/importer/import-press-release.js
- tools/importer/parsers/hero-article.js
- tools/importer/reports/import-featured-story.report.xlsx
- tools/importer/urls-fs4.txt
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-featured-story.report.xlsx
+++ b/tools/importer/reports/import-featured-story.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="61">
   <si>
     <t>_reportFile</t>
   </si>
@@ -152,16 +152,55 @@
     <t>workspace/migration-work/pages/featured-story-4.report.json</t>
   </si>
   <si>
+    <t>["hero-article","cards-news"]</t>
+  </si>
+  <si>
     <t>workspace/migration-work/pages/featured-story-4</t>
   </si>
   <si>
-    <t>2026-04-16T08:05:17.099Z</t>
+    <t>2026-04-16T08:37:23.680Z</t>
   </si>
   <si>
     <t>Get Ahead with Energy Storage or Risk Getting Left Behind | Honeywell</t>
   </si>
   <si>
     <t>file:///workspace/migration-work/pages/featured-story-4.html</t>
+  </si>
+  <si>
+    <t>workspace/migration-work/pages/press-release-1.report.json</t>
+  </si>
+  <si>
+    <t>["hero-corporate"]</t>
+  </si>
+  <si>
+    <t>workspace/migration-work/pages/press-release-1</t>
+  </si>
+  <si>
+    <t>press-release</t>
+  </si>
+  <si>
+    <t>2026-04-16T08:05:22.255Z</t>
+  </si>
+  <si>
+    <t>Honeywell to Help Dangote Double Production Capabilities at Africa’s Largest Refinery</t>
+  </si>
+  <si>
+    <t>file:///workspace/migration-work/pages/press-release-1.html</t>
+  </si>
+  <si>
+    <t>workspace/migration-work/pages/press-release-2.report.json</t>
+  </si>
+  <si>
+    <t>workspace/migration-work/pages/press-release-2</t>
+  </si>
+  <si>
+    <t>2026-04-16T08:05:29.010Z</t>
+  </si>
+  <si>
+    <t>Honeywell Carbon Capture Technology to Help Transform Shuttered Power Plant Into Fertilizer Facility Supporting U.S. Farmers</t>
+  </si>
+  <si>
+    <t>file:///workspace/migration-work/pages/press-release-2.html</t>
   </si>
 </sst>
 </file>
@@ -550,7 +589,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="50" customWidth="1"/>
@@ -757,7 +796,7 @@
         <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
         <v>11</v>
@@ -766,7 +805,7 @@
         <v>11</v>
       </c>
       <c r="E7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F7" t="s">
         <v>21</v>
@@ -775,13 +814,77 @@
         <v>29</v>
       </c>
       <c r="H7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="J7" t="s">
-        <v>47</v>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H8" t="s">
+        <v>53</v>
+      </c>
+      <c r="I8" t="s">
+        <v>54</v>
+      </c>
+      <c r="J8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B9" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>57</v>
+      </c>
+      <c r="F9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G9" t="s">
+        <v>52</v>
+      </c>
+      <c r="H9" t="s">
+        <v>58</v>
+      </c>
+      <c r="I9" t="s">
+        <v>59</v>
+      </c>
+      <c r="J9" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>